<commit_message>
decimal no, changes in govt plot
</commit_message>
<xml_diff>
--- a/uploads/forest_land_excels/Non-forest_land_(1).xlsx
+++ b/uploads/forest_land_excels/Non-forest_land_(1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maasuser\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C894680-B1C0-4E71-8FAE-B1F0510CD394}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC1D0E30-0551-4CDA-9210-9DFCD01BD8E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="45">
   <si>
     <t>District</t>
   </si>
@@ -530,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDAB6792-0B21-42AB-8D6E-80AC551EBBEA}">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="13.28515625" customWidth="1"/>
@@ -579,45 +579,45 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1">
+        <v>102</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" s="1">
+        <v>8.75</v>
+      </c>
+      <c r="K2" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -625,71 +625,33 @@
         <v>10</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E3" s="1">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="J3" s="1">
-        <v>8.75</v>
+        <v>6.3</v>
       </c>
       <c r="K3" s="1">
-        <v>6.5</v>
+        <v>5.2</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="1">
-        <v>118</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J4" s="1">
-        <v>6.3</v>
-      </c>
-      <c r="K4" s="1">
-        <v>5.2</v>
-      </c>
-      <c r="L4" s="1" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>